<commit_message>
refactor(assay): drop has sample (#30)
* refactor(assay): drop redundant has_sample property

* refactor(assay): drop ordering and allow EFO on sample_processing

* chore: regen

* docs(readme): update toplevel diagram
</commit_message>
<xml_diff>
--- a/project/excel/modos_schema.xlsx
+++ b/project/excel/modos_schema.xlsx
@@ -649,49 +649,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>has_sample</t>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>has_data</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>has_data</t>
+          <t>omics_type</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>omics_type</t>
+          <t>sample_processing</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>sample_processing</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>name</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
           <t>description</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"GENOMICS,TRANSCRIPTOMICS,METABOLOMICS,PROTEOMICS"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>